<commit_message>
docs: fyll i offpist-underlaget (ja/nej-varden, nivaspann och regel)
Underlag: offpistTillgang, glaciarakning och guideverksamhet ifyllda
(ja/nej) och offpistNivaMin/Max (tal 1-5) for alla 15 orter, avstamda
mot texterna pa Anteckningar. offpistNote ar fortfarande tom.

Regel for spannet inskriven i markdown-mallen och pa Definitioner: Max
raknar in all terrang som nas fran orten (aven turakning, heliskiing och
guidad glaciarakning), Min ar aldrig 1 om orten har offpist.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/offpist-underlag.xlsx
+++ b/docs/offpist-underlag.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User1\AppData\Local\Temp\claude\C--Users-User1-Downloads-project-bolt-sb1-qfebkjhm-project\b978087f-0d86-4b0b-9125-95908213e11f\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDB7537-AAF9-4041-BC92-F5E2C2C922B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD30759-837A-4C64-8B07-7A81041AC2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Underlag" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="163">
   <si>
     <t>id</t>
   </si>
@@ -499,6 +499,18 @@
   </si>
   <si>
     <t>Underlaget kommer från lokala bergsguider och är granskat. Informationen är vägledande - all offpiståkning sker på eget ansvar, och varje åkare ansvarar själv för lavinbedömning, utrustning och terrängval.</t>
+  </si>
+  <si>
+    <t>ja</t>
+  </si>
+  <si>
+    <t>nej</t>
+  </si>
+  <si>
+    <t>Regel: offpistNivaMax räknar in all terräng som nås från orten, även turåkning, heliskiing och guidad glaciäråkning.</t>
+  </si>
+  <si>
+    <t>offpistNivaMin är den lugnaste meningsfulla offpistterrängen, aldrig 1 om orten har offpist alls.</t>
   </si>
 </sst>
 </file>
@@ -940,6 +952,30 @@
       <c r="B2" t="s">
         <v>12</v>
       </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>159</v>
+      </c>
+      <c r="F2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G2" t="s">
+        <v>159</v>
+      </c>
+      <c r="H2" t="s">
+        <v>159</v>
+      </c>
+      <c r="I2" t="s">
+        <v>160</v>
+      </c>
+      <c r="J2" t="s">
+        <v>159</v>
+      </c>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
@@ -949,6 +985,30 @@
       <c r="B3" t="s">
         <v>14</v>
       </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G3" t="s">
+        <v>159</v>
+      </c>
+      <c r="H3" t="s">
+        <v>159</v>
+      </c>
+      <c r="I3" t="s">
+        <v>160</v>
+      </c>
+      <c r="J3" t="s">
+        <v>159</v>
+      </c>
       <c r="K3" s="2"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
@@ -958,6 +1018,30 @@
       <c r="B4" t="s">
         <v>16</v>
       </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4" t="s">
+        <v>159</v>
+      </c>
+      <c r="F4" t="s">
+        <v>159</v>
+      </c>
+      <c r="G4" t="s">
+        <v>159</v>
+      </c>
+      <c r="H4" t="s">
+        <v>159</v>
+      </c>
+      <c r="I4" t="s">
+        <v>159</v>
+      </c>
+      <c r="J4" t="s">
+        <v>159</v>
+      </c>
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
@@ -967,6 +1051,30 @@
       <c r="B5" t="s">
         <v>18</v>
       </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F5" t="s">
+        <v>159</v>
+      </c>
+      <c r="G5" t="s">
+        <v>159</v>
+      </c>
+      <c r="H5" t="s">
+        <v>159</v>
+      </c>
+      <c r="I5" t="s">
+        <v>160</v>
+      </c>
+      <c r="J5" t="s">
+        <v>159</v>
+      </c>
       <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
@@ -976,6 +1084,30 @@
       <c r="B6" t="s">
         <v>20</v>
       </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6" t="s">
+        <v>159</v>
+      </c>
+      <c r="F6" t="s">
+        <v>159</v>
+      </c>
+      <c r="G6" t="s">
+        <v>159</v>
+      </c>
+      <c r="H6" t="s">
+        <v>159</v>
+      </c>
+      <c r="I6" t="s">
+        <v>160</v>
+      </c>
+      <c r="J6" t="s">
+        <v>159</v>
+      </c>
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
@@ -985,6 +1117,30 @@
       <c r="B7" t="s">
         <v>22</v>
       </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>159</v>
+      </c>
+      <c r="F7" t="s">
+        <v>159</v>
+      </c>
+      <c r="G7" t="s">
+        <v>159</v>
+      </c>
+      <c r="H7" t="s">
+        <v>160</v>
+      </c>
+      <c r="I7" t="s">
+        <v>160</v>
+      </c>
+      <c r="J7" t="s">
+        <v>159</v>
+      </c>
       <c r="K7" s="2"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
@@ -994,6 +1150,30 @@
       <c r="B8" t="s">
         <v>24</v>
       </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8" t="s">
+        <v>159</v>
+      </c>
+      <c r="F8" t="s">
+        <v>159</v>
+      </c>
+      <c r="G8" t="s">
+        <v>159</v>
+      </c>
+      <c r="H8" t="s">
+        <v>159</v>
+      </c>
+      <c r="I8" t="s">
+        <v>160</v>
+      </c>
+      <c r="J8" t="s">
+        <v>159</v>
+      </c>
       <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
@@ -1003,6 +1183,30 @@
       <c r="B9" t="s">
         <v>26</v>
       </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+      <c r="E9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F9" t="s">
+        <v>159</v>
+      </c>
+      <c r="G9" t="s">
+        <v>159</v>
+      </c>
+      <c r="H9" t="s">
+        <v>159</v>
+      </c>
+      <c r="I9" t="s">
+        <v>159</v>
+      </c>
+      <c r="J9" t="s">
+        <v>159</v>
+      </c>
       <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
@@ -1012,6 +1216,30 @@
       <c r="B10" t="s">
         <v>28</v>
       </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+      <c r="E10" t="s">
+        <v>159</v>
+      </c>
+      <c r="F10" t="s">
+        <v>159</v>
+      </c>
+      <c r="G10" t="s">
+        <v>159</v>
+      </c>
+      <c r="H10" t="s">
+        <v>159</v>
+      </c>
+      <c r="I10" t="s">
+        <v>160</v>
+      </c>
+      <c r="J10" t="s">
+        <v>159</v>
+      </c>
       <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
@@ -1021,6 +1249,30 @@
       <c r="B11" t="s">
         <v>30</v>
       </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11" t="s">
+        <v>159</v>
+      </c>
+      <c r="F11" t="s">
+        <v>159</v>
+      </c>
+      <c r="G11" t="s">
+        <v>159</v>
+      </c>
+      <c r="H11" t="s">
+        <v>159</v>
+      </c>
+      <c r="I11" t="s">
+        <v>160</v>
+      </c>
+      <c r="J11" t="s">
+        <v>159</v>
+      </c>
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
@@ -1030,6 +1282,30 @@
       <c r="B12" t="s">
         <v>32</v>
       </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12" t="s">
+        <v>159</v>
+      </c>
+      <c r="F12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G12" t="s">
+        <v>159</v>
+      </c>
+      <c r="H12" t="s">
+        <v>159</v>
+      </c>
+      <c r="I12" t="s">
+        <v>160</v>
+      </c>
+      <c r="J12" t="s">
+        <v>159</v>
+      </c>
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
@@ -1039,6 +1315,30 @@
       <c r="B13" t="s">
         <v>34</v>
       </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13" t="s">
+        <v>159</v>
+      </c>
+      <c r="F13" t="s">
+        <v>159</v>
+      </c>
+      <c r="G13" t="s">
+        <v>159</v>
+      </c>
+      <c r="H13" t="s">
+        <v>159</v>
+      </c>
+      <c r="I13" t="s">
+        <v>160</v>
+      </c>
+      <c r="J13" t="s">
+        <v>159</v>
+      </c>
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
@@ -1048,6 +1348,30 @@
       <c r="B14" t="s">
         <v>36</v>
       </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+      <c r="D14">
+        <v>5</v>
+      </c>
+      <c r="E14" t="s">
+        <v>159</v>
+      </c>
+      <c r="F14" t="s">
+        <v>159</v>
+      </c>
+      <c r="G14" t="s">
+        <v>159</v>
+      </c>
+      <c r="H14" t="s">
+        <v>159</v>
+      </c>
+      <c r="I14" t="s">
+        <v>160</v>
+      </c>
+      <c r="J14" t="s">
+        <v>159</v>
+      </c>
       <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
@@ -1057,6 +1381,30 @@
       <c r="B15" t="s">
         <v>38</v>
       </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15" t="s">
+        <v>159</v>
+      </c>
+      <c r="F15" t="s">
+        <v>160</v>
+      </c>
+      <c r="G15" t="s">
+        <v>159</v>
+      </c>
+      <c r="H15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I15" t="s">
+        <v>160</v>
+      </c>
+      <c r="J15" t="s">
+        <v>159</v>
+      </c>
       <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
@@ -1065,6 +1413,30 @@
       </c>
       <c r="B16" t="s">
         <v>40</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>159</v>
+      </c>
+      <c r="F16" t="s">
+        <v>159</v>
+      </c>
+      <c r="G16" t="s">
+        <v>159</v>
+      </c>
+      <c r="H16" t="s">
+        <v>159</v>
+      </c>
+      <c r="I16" t="s">
+        <v>160</v>
+      </c>
+      <c r="J16" t="s">
+        <v>159</v>
       </c>
       <c r="K16" s="2"/>
     </row>
@@ -1083,7 +1455,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1116,110 +1488,120 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>45</v>
+      <c r="A7" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" t="s">
-        <v>47</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" t="s">
-        <v>49</v>
+      <c r="A9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>54</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B14" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" t="s">
-        <v>60</v>
+      <c r="A18" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>7</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B22" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>63</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: offpistNote ifyllt och ansvarsfriskrivningen andrad i offpist-underlaget
offpistNote (max 140 tecken, byggda enbart pa Anteckningar-texterna) for
alla 15 orter. Ansvarsfriskrivningen pa Definitioner anger nu att
underlaget saknar verifierad kalla istallet for att det ar granskat av
bergsguider.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/offpist-underlag.xlsx
+++ b/docs/offpist-underlag.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User1\AppData\Local\Temp\claude\C--Users-User1-Downloads-project-bolt-sb1-qfebkjhm-project\b978087f-0d86-4b0b-9125-95908213e11f\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD30759-837A-4C64-8B07-7A81041AC2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169838F5-76BA-4387-AD29-6E5075562704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="178">
   <si>
     <t>id</t>
   </si>
@@ -498,9 +498,6 @@
     <t>Ansvarsfriskrivning</t>
   </si>
   <si>
-    <t>Underlaget kommer från lokala bergsguider och är granskat. Informationen är vägledande - all offpiståkning sker på eget ansvar, och varje åkare ansvarar själv för lavinbedömning, utrustning och terrängval.</t>
-  </si>
-  <si>
     <t>ja</t>
   </si>
   <si>
@@ -511,6 +508,54 @@
   </si>
   <si>
     <t>offpistNivaMin är den lugnaste meningsfulla offpistterrängen, aldrig 1 om orten har offpist alls.</t>
+  </si>
+  <si>
+    <t>Liftnära puderfält vid Chanrossa och ytor runt Loze Express, Freeride Lab ca 15 min gång; Gébroulaz-glaciären kräver guide.</t>
+  </si>
+  <si>
+    <t>Skogsåkning bland lärkträd i Les Arcs, baksidan av Aiguille Rouge efter kort hike; Bellecôtes norrsida farlig utan lokalkännedom.</t>
+  </si>
+  <si>
+    <t>Liftnära freeride vid Le Fornet, Toviere och Grande Motte; glaciärerna och de branta couloirerna kräver guide.</t>
+  </si>
+  <si>
+    <t>Trädåkning runt Morzine och Les Gets vid dålig sikt; korta stigningar vid Pointe de Mossettes når puder över schweiziska gränsen.</t>
+  </si>
+  <si>
+    <t>Combe de Gers i Flaine har brant nordsnö; lapiaz (dolda kalkstenssprickor) gör ofta guide till krav i stora delar av Flaine.</t>
+  </si>
+  <si>
+    <t>Snällare, böljande öppna fält och lättvandrade kammar; ofta folktom turåkning som passar nybörjare på stighudar.</t>
+  </si>
+  <si>
+    <t>Från Pic Blanc (3330 m) nås Grand Sablat och Combe du Loup; guide rekommenderas starkt för baksidesåken ner mot dalen.</t>
+  </si>
+  <si>
+    <t>Gles lärkskog med trädåkning i toppklass, kalfjäll vid L'Eychauda, kort stigning till Cucumelle; guide rekommenderas för Ecrins-turer.</t>
+  </si>
+  <si>
+    <t>Skogsåkning bland granar runt Cote 2000; vandring mot Mont Joly når brantare rännor på baksidan, där guide är ett absolut krav.</t>
+  </si>
+  <si>
+    <t>Brant liftnära offpist vid Grands Montets; glaciärerna har dolda sprickor och Vallée Blanche ska göras med utbildad bergsguide.</t>
+  </si>
+  <si>
+    <t>Retour d'Est ger ofta mycket snö på franska sidan; branta åk från Mount Chaberton, guide ovärderlig på italienska sidan.</t>
+  </si>
+  <si>
+    <t>Mont Valaisan ger systemets bästa offpist efter kort tur; heliskiing mot Ruitor-glaciären vid italienska gränsen kräver guide.</t>
+  </si>
+  <si>
+    <t>Snäll, vindskyddad terräng bland snötunga granar och öppna fält – bra för offpistnybörjare och för att lära sig turåkning.</t>
+  </si>
+  <si>
+    <t>Stor fallhöjd och länge orörd snö i gles skog och kalfjäll; gränsar till Vanoise, där guide rekommenderas för toppturer.</t>
+  </si>
+  <si>
+    <t>Offpist i La Fée-sektorn; övergången till grannorten La Grave kräver i princip guide – opistad extremterräng och glaciärsprickor.</t>
+  </si>
+  <si>
+    <t>Underlaget är sammanställt av projektet och har ännu ingen verifierad källa. Informationen är vägledande - all offpiståkning sker på eget ansvar, och varje åkare ansvarar själv för lavinbedömning, utrustning och terrängval.</t>
   </si>
 </sst>
 </file>
@@ -945,7 +990,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -959,26 +1004,28 @@
         <v>5</v>
       </c>
       <c r="E2" t="s">
+        <v>158</v>
+      </c>
+      <c r="F2" t="s">
+        <v>158</v>
+      </c>
+      <c r="G2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H2" t="s">
+        <v>158</v>
+      </c>
+      <c r="I2" t="s">
         <v>159</v>
       </c>
-      <c r="F2" t="s">
-        <v>159</v>
-      </c>
-      <c r="G2" t="s">
-        <v>159</v>
-      </c>
-      <c r="H2" t="s">
-        <v>159</v>
-      </c>
-      <c r="I2" t="s">
-        <v>160</v>
-      </c>
       <c r="J2" t="s">
-        <v>159</v>
-      </c>
-      <c r="K2" s="2"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -992,26 +1039,28 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G3" t="s">
+        <v>158</v>
+      </c>
+      <c r="H3" t="s">
+        <v>158</v>
+      </c>
+      <c r="I3" t="s">
         <v>159</v>
       </c>
-      <c r="F3" t="s">
-        <v>159</v>
-      </c>
-      <c r="G3" t="s">
-        <v>159</v>
-      </c>
-      <c r="H3" t="s">
-        <v>159</v>
-      </c>
-      <c r="I3" t="s">
-        <v>160</v>
-      </c>
       <c r="J3" t="s">
-        <v>159</v>
-      </c>
-      <c r="K3" s="2"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1025,26 +1074,28 @@
         <v>5</v>
       </c>
       <c r="E4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J4" t="s">
-        <v>159</v>
-      </c>
-      <c r="K4" s="2"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1058,26 +1109,28 @@
         <v>4</v>
       </c>
       <c r="E5" t="s">
+        <v>158</v>
+      </c>
+      <c r="F5" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" t="s">
+        <v>158</v>
+      </c>
+      <c r="H5" t="s">
+        <v>158</v>
+      </c>
+      <c r="I5" t="s">
         <v>159</v>
       </c>
-      <c r="F5" t="s">
-        <v>159</v>
-      </c>
-      <c r="G5" t="s">
-        <v>159</v>
-      </c>
-      <c r="H5" t="s">
-        <v>159</v>
-      </c>
-      <c r="I5" t="s">
-        <v>160</v>
-      </c>
       <c r="J5" t="s">
-        <v>159</v>
-      </c>
-      <c r="K5" s="2"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1091,26 +1144,28 @@
         <v>4</v>
       </c>
       <c r="E6" t="s">
+        <v>158</v>
+      </c>
+      <c r="F6" t="s">
+        <v>158</v>
+      </c>
+      <c r="G6" t="s">
+        <v>158</v>
+      </c>
+      <c r="H6" t="s">
+        <v>158</v>
+      </c>
+      <c r="I6" t="s">
         <v>159</v>
       </c>
-      <c r="F6" t="s">
-        <v>159</v>
-      </c>
-      <c r="G6" t="s">
-        <v>159</v>
-      </c>
-      <c r="H6" t="s">
-        <v>159</v>
-      </c>
-      <c r="I6" t="s">
-        <v>160</v>
-      </c>
       <c r="J6" t="s">
-        <v>159</v>
-      </c>
-      <c r="K6" s="2"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1124,26 +1179,28 @@
         <v>3</v>
       </c>
       <c r="E7" t="s">
+        <v>158</v>
+      </c>
+      <c r="F7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G7" t="s">
+        <v>158</v>
+      </c>
+      <c r="H7" t="s">
         <v>159</v>
       </c>
-      <c r="F7" t="s">
+      <c r="I7" t="s">
         <v>159</v>
       </c>
-      <c r="G7" t="s">
-        <v>159</v>
-      </c>
-      <c r="H7" t="s">
-        <v>160</v>
-      </c>
-      <c r="I7" t="s">
-        <v>160</v>
-      </c>
       <c r="J7" t="s">
-        <v>159</v>
-      </c>
-      <c r="K7" s="2"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -1157,26 +1214,28 @@
         <v>5</v>
       </c>
       <c r="E8" t="s">
+        <v>158</v>
+      </c>
+      <c r="F8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G8" t="s">
+        <v>158</v>
+      </c>
+      <c r="H8" t="s">
+        <v>158</v>
+      </c>
+      <c r="I8" t="s">
         <v>159</v>
       </c>
-      <c r="F8" t="s">
-        <v>159</v>
-      </c>
-      <c r="G8" t="s">
-        <v>159</v>
-      </c>
-      <c r="H8" t="s">
-        <v>159</v>
-      </c>
-      <c r="I8" t="s">
-        <v>160</v>
-      </c>
       <c r="J8" t="s">
-        <v>159</v>
-      </c>
-      <c r="K8" s="2"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -1190,26 +1249,28 @@
         <v>5</v>
       </c>
       <c r="E9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J9" t="s">
-        <v>159</v>
-      </c>
-      <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -1223,26 +1284,28 @@
         <v>5</v>
       </c>
       <c r="E10" t="s">
+        <v>158</v>
+      </c>
+      <c r="F10" t="s">
+        <v>158</v>
+      </c>
+      <c r="G10" t="s">
+        <v>158</v>
+      </c>
+      <c r="H10" t="s">
+        <v>158</v>
+      </c>
+      <c r="I10" t="s">
         <v>159</v>
       </c>
-      <c r="F10" t="s">
-        <v>159</v>
-      </c>
-      <c r="G10" t="s">
-        <v>159</v>
-      </c>
-      <c r="H10" t="s">
-        <v>159</v>
-      </c>
-      <c r="I10" t="s">
-        <v>160</v>
-      </c>
       <c r="J10" t="s">
-        <v>159</v>
-      </c>
-      <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -1256,26 +1319,28 @@
         <v>4</v>
       </c>
       <c r="E11" t="s">
+        <v>158</v>
+      </c>
+      <c r="F11" t="s">
+        <v>158</v>
+      </c>
+      <c r="G11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H11" t="s">
+        <v>158</v>
+      </c>
+      <c r="I11" t="s">
         <v>159</v>
       </c>
-      <c r="F11" t="s">
-        <v>159</v>
-      </c>
-      <c r="G11" t="s">
-        <v>159</v>
-      </c>
-      <c r="H11" t="s">
-        <v>159</v>
-      </c>
-      <c r="I11" t="s">
-        <v>160</v>
-      </c>
       <c r="J11" t="s">
-        <v>159</v>
-      </c>
-      <c r="K11" s="2"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -1289,26 +1354,28 @@
         <v>5</v>
       </c>
       <c r="E12" t="s">
+        <v>158</v>
+      </c>
+      <c r="F12" t="s">
+        <v>158</v>
+      </c>
+      <c r="G12" t="s">
+        <v>158</v>
+      </c>
+      <c r="H12" t="s">
+        <v>158</v>
+      </c>
+      <c r="I12" t="s">
         <v>159</v>
       </c>
-      <c r="F12" t="s">
-        <v>159</v>
-      </c>
-      <c r="G12" t="s">
-        <v>159</v>
-      </c>
-      <c r="H12" t="s">
-        <v>159</v>
-      </c>
-      <c r="I12" t="s">
-        <v>160</v>
-      </c>
       <c r="J12" t="s">
-        <v>159</v>
-      </c>
-      <c r="K12" s="2"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -1322,26 +1389,28 @@
         <v>4</v>
       </c>
       <c r="E13" t="s">
+        <v>158</v>
+      </c>
+      <c r="F13" t="s">
+        <v>158</v>
+      </c>
+      <c r="G13" t="s">
+        <v>158</v>
+      </c>
+      <c r="H13" t="s">
+        <v>158</v>
+      </c>
+      <c r="I13" t="s">
         <v>159</v>
       </c>
-      <c r="F13" t="s">
-        <v>159</v>
-      </c>
-      <c r="G13" t="s">
-        <v>159</v>
-      </c>
-      <c r="H13" t="s">
-        <v>159</v>
-      </c>
-      <c r="I13" t="s">
-        <v>160</v>
-      </c>
       <c r="J13" t="s">
-        <v>159</v>
-      </c>
-      <c r="K13" s="2"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>35</v>
       </c>
@@ -1355,26 +1424,28 @@
         <v>5</v>
       </c>
       <c r="E14" t="s">
+        <v>158</v>
+      </c>
+      <c r="F14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G14" t="s">
+        <v>158</v>
+      </c>
+      <c r="H14" t="s">
+        <v>158</v>
+      </c>
+      <c r="I14" t="s">
         <v>159</v>
       </c>
-      <c r="F14" t="s">
-        <v>159</v>
-      </c>
-      <c r="G14" t="s">
-        <v>159</v>
-      </c>
-      <c r="H14" t="s">
-        <v>159</v>
-      </c>
-      <c r="I14" t="s">
-        <v>160</v>
-      </c>
       <c r="J14" t="s">
-        <v>159</v>
-      </c>
-      <c r="K14" s="2"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -1388,26 +1459,28 @@
         <v>3</v>
       </c>
       <c r="E15" t="s">
+        <v>158</v>
+      </c>
+      <c r="F15" t="s">
         <v>159</v>
       </c>
-      <c r="F15" t="s">
-        <v>160</v>
-      </c>
       <c r="G15" t="s">
+        <v>158</v>
+      </c>
+      <c r="H15" t="s">
         <v>159</v>
       </c>
-      <c r="H15" t="s">
-        <v>160</v>
-      </c>
       <c r="I15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J15" t="s">
-        <v>159</v>
-      </c>
-      <c r="K15" s="2"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -1421,24 +1494,26 @@
         <v>5</v>
       </c>
       <c r="E16" t="s">
+        <v>158</v>
+      </c>
+      <c r="F16" t="s">
+        <v>158</v>
+      </c>
+      <c r="G16" t="s">
+        <v>158</v>
+      </c>
+      <c r="H16" t="s">
+        <v>158</v>
+      </c>
+      <c r="I16" t="s">
         <v>159</v>
       </c>
-      <c r="F16" t="s">
-        <v>159</v>
-      </c>
-      <c r="G16" t="s">
-        <v>159</v>
-      </c>
-      <c r="H16" t="s">
-        <v>159</v>
-      </c>
-      <c r="I16" t="s">
-        <v>160</v>
-      </c>
       <c r="J16" t="s">
-        <v>159</v>
-      </c>
-      <c r="K16" s="2"/>
+        <v>158</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>175</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -1469,7 +1544,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1489,12 +1564,12 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>